<commit_message>
CodeWeek ana sayfası, ekleyenler listesi, skor tablosu ve yeni terim görselleri
- Başlık: Bilişime İlk Adım / Terimler Sözlüğü; slogan ve ana sayfa metni CodeWeek için güncellendi
- Terim eklerken ad soyad ve okul zorunlu; ekleyen sözlükte görünür (üyelik yok)
- Kart yap kutusu yerine Sözlüğe ekleyenler listesi
- En yüksek skorlar veritabanında tutulur (/api/scores)
- Güvenli internet ve bilişim hukuku terim görselleri

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gorsel-istemleri.xlsx
+++ b/gorsel-istemleri.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC680FF3-11B8-4577-81A6-B2F3F84CB230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FAC3829-F69E-4838-B015-519FBCFB44CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28005" yWindow="2940" windowWidth="23430" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="16200" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Terim görselleri" sheetId="1" r:id="rId1"/>
@@ -3376,9 +3376,6 @@
 Show a concrete, easy-to-read scene that lets a high school student guess the concept, rather than abstract symbols.</t>
   </si>
   <si>
-    <t>test-verisi.png</t>
-  </si>
-  <si>
     <t>Test verisi</t>
   </si>
   <si>
@@ -5720,6 +5717,9 @@
     <t>Square 1:1 image. Clean, modern editorial tech illustration with soft depth and gentle gradients; deep navy, teal and a warm red (#c4161c) accent on a light background; one clear focal idea; friendly and school-appropriate; any people are teenagers or adults. Absolutely no text, letters, numbers, logos, brand marks or watermarks.
 Illustrate the technical term "Shader" (Gölgelendirici) from the field of "Oyun Tasarımı". Meaning (Turkish): Bir yüzeyin ekranda nasıl görüneceğini hesaplayan program. More context (Turkish): Işık, renk, parlaklık, saydamlık ve özel efektleri belirler; ekran kartında çalışır.
 Show a concrete, easy-to-read scene that +E49lets a high school student guess the concept, rather than abstract symbols.</t>
+  </si>
+  <si>
+    <t>.png</t>
   </si>
 </sst>
 </file>
@@ -6943,7 +6943,7 @@
         <v>122</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>1557</v>
+        <v>1556</v>
       </c>
     </row>
     <row r="49" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
@@ -10279,19 +10279,19 @@
       </c>
     </row>
     <row r="245" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
-      <c r="A245" s="2" t="s">
+      <c r="A245" s="3" t="s">
         <v>745</v>
       </c>
-      <c r="B245" s="2" t="s">
+      <c r="B245" s="3" t="s">
         <v>746</v>
       </c>
-      <c r="C245" s="2" t="s">
+      <c r="C245" s="3" t="s">
         <v>722</v>
       </c>
-      <c r="D245" s="2" t="s">
+      <c r="D245" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="E245" s="2" t="s">
+      <c r="E245" s="3" t="s">
         <v>747</v>
       </c>
     </row>
@@ -10636,19 +10636,19 @@
       </c>
     </row>
     <row r="266" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
-      <c r="A266" s="2" t="s">
+      <c r="A266" s="3" t="s">
         <v>808</v>
       </c>
-      <c r="B266" s="2" t="s">
+      <c r="B266" s="3" t="s">
         <v>809</v>
       </c>
-      <c r="C266" s="2" t="s">
+      <c r="C266" s="3" t="s">
         <v>722</v>
       </c>
-      <c r="D266" s="2" t="s">
+      <c r="D266" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="E266" s="2" t="s">
+      <c r="E266" s="3" t="s">
         <v>810</v>
       </c>
     </row>
@@ -11146,19 +11146,19 @@
       </c>
     </row>
     <row r="296" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
-      <c r="A296" s="2" t="s">
+      <c r="A296" s="3" t="s">
         <v>899</v>
       </c>
-      <c r="B296" s="2" t="s">
+      <c r="B296" s="3" t="s">
         <v>900</v>
       </c>
-      <c r="C296" s="2" t="s">
+      <c r="C296" s="3" t="s">
         <v>813</v>
       </c>
-      <c r="D296" s="2" t="s">
+      <c r="D296" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E296" s="2" t="s">
+      <c r="E296" s="3" t="s">
         <v>901</v>
       </c>
     </row>
@@ -11249,10 +11249,10 @@
     </row>
     <row r="302" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A302" s="2" t="s">
+        <v>1557</v>
+      </c>
+      <c r="B302" s="2" t="s">
         <v>918</v>
-      </c>
-      <c r="B302" s="2" t="s">
-        <v>919</v>
       </c>
       <c r="C302" s="2" t="s">
         <v>904</v>
@@ -11261,15 +11261,15 @@
         <v>79</v>
       </c>
       <c r="E302" s="2" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
     </row>
     <row r="303" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A303" s="2" t="s">
+        <v>920</v>
+      </c>
+      <c r="B303" s="2" t="s">
         <v>921</v>
-      </c>
-      <c r="B303" s="2" t="s">
-        <v>922</v>
       </c>
       <c r="C303" s="2" t="s">
         <v>904</v>
@@ -11278,15 +11278,15 @@
         <v>79</v>
       </c>
       <c r="E303" s="2" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
     </row>
     <row r="304" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A304" s="2" t="s">
+        <v>923</v>
+      </c>
+      <c r="B304" s="2" t="s">
         <v>924</v>
-      </c>
-      <c r="B304" s="2" t="s">
-        <v>925</v>
       </c>
       <c r="C304" s="2" t="s">
         <v>904</v>
@@ -11295,15 +11295,15 @@
         <v>79</v>
       </c>
       <c r="E304" s="2" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
     </row>
     <row r="305" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A305" s="2" t="s">
+        <v>926</v>
+      </c>
+      <c r="B305" s="2" t="s">
         <v>927</v>
-      </c>
-      <c r="B305" s="2" t="s">
-        <v>928</v>
       </c>
       <c r="C305" s="2" t="s">
         <v>904</v>
@@ -11312,15 +11312,15 @@
         <v>79</v>
       </c>
       <c r="E305" s="2" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
     </row>
     <row r="306" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A306" s="2" t="s">
+        <v>929</v>
+      </c>
+      <c r="B306" s="2" t="s">
         <v>930</v>
-      </c>
-      <c r="B306" s="2" t="s">
-        <v>931</v>
       </c>
       <c r="C306" s="2" t="s">
         <v>904</v>
@@ -11329,15 +11329,15 @@
         <v>79</v>
       </c>
       <c r="E306" s="2" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
     </row>
     <row r="307" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A307" s="2" t="s">
+        <v>932</v>
+      </c>
+      <c r="B307" s="2" t="s">
         <v>933</v>
-      </c>
-      <c r="B307" s="2" t="s">
-        <v>934</v>
       </c>
       <c r="C307" s="2" t="s">
         <v>904</v>
@@ -11346,15 +11346,15 @@
         <v>79</v>
       </c>
       <c r="E307" s="2" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
     </row>
     <row r="308" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A308" s="2" t="s">
+        <v>935</v>
+      </c>
+      <c r="B308" s="2" t="s">
         <v>936</v>
-      </c>
-      <c r="B308" s="2" t="s">
-        <v>937</v>
       </c>
       <c r="C308" s="2" t="s">
         <v>904</v>
@@ -11363,15 +11363,15 @@
         <v>79</v>
       </c>
       <c r="E308" s="2" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
     </row>
     <row r="309" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A309" s="2" t="s">
+        <v>938</v>
+      </c>
+      <c r="B309" s="2" t="s">
         <v>939</v>
-      </c>
-      <c r="B309" s="2" t="s">
-        <v>940</v>
       </c>
       <c r="C309" s="2" t="s">
         <v>904</v>
@@ -11380,15 +11380,15 @@
         <v>79</v>
       </c>
       <c r="E309" s="2" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
     </row>
     <row r="310" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A310" s="2" t="s">
+        <v>941</v>
+      </c>
+      <c r="B310" s="2" t="s">
         <v>942</v>
-      </c>
-      <c r="B310" s="2" t="s">
-        <v>943</v>
       </c>
       <c r="C310" s="2" t="s">
         <v>904</v>
@@ -11397,15 +11397,15 @@
         <v>79</v>
       </c>
       <c r="E310" s="2" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
     </row>
     <row r="311" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A311" s="2" t="s">
+        <v>944</v>
+      </c>
+      <c r="B311" s="2" t="s">
         <v>945</v>
-      </c>
-      <c r="B311" s="2" t="s">
-        <v>946</v>
       </c>
       <c r="C311" s="2" t="s">
         <v>904</v>
@@ -11414,15 +11414,15 @@
         <v>122</v>
       </c>
       <c r="E311" s="2" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
     </row>
     <row r="312" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A312" s="2" t="s">
+        <v>947</v>
+      </c>
+      <c r="B312" s="2" t="s">
         <v>948</v>
-      </c>
-      <c r="B312" s="2" t="s">
-        <v>949</v>
       </c>
       <c r="C312" s="2" t="s">
         <v>904</v>
@@ -11431,15 +11431,15 @@
         <v>79</v>
       </c>
       <c r="E312" s="2" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
     </row>
     <row r="313" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A313" s="2" t="s">
+        <v>950</v>
+      </c>
+      <c r="B313" s="2" t="s">
         <v>951</v>
-      </c>
-      <c r="B313" s="2" t="s">
-        <v>952</v>
       </c>
       <c r="C313" s="2" t="s">
         <v>904</v>
@@ -11448,15 +11448,15 @@
         <v>122</v>
       </c>
       <c r="E313" s="2" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
     </row>
     <row r="314" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A314" s="2" t="s">
+        <v>953</v>
+      </c>
+      <c r="B314" s="2" t="s">
         <v>954</v>
-      </c>
-      <c r="B314" s="2" t="s">
-        <v>955</v>
       </c>
       <c r="C314" s="2" t="s">
         <v>904</v>
@@ -11465,15 +11465,15 @@
         <v>79</v>
       </c>
       <c r="E314" s="2" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
     </row>
     <row r="315" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A315" s="2" t="s">
+        <v>956</v>
+      </c>
+      <c r="B315" s="2" t="s">
         <v>957</v>
-      </c>
-      <c r="B315" s="2" t="s">
-        <v>958</v>
       </c>
       <c r="C315" s="2" t="s">
         <v>904</v>
@@ -11482,15 +11482,15 @@
         <v>79</v>
       </c>
       <c r="E315" s="2" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
     </row>
     <row r="316" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A316" s="2" t="s">
+        <v>959</v>
+      </c>
+      <c r="B316" s="2" t="s">
         <v>960</v>
-      </c>
-      <c r="B316" s="2" t="s">
-        <v>961</v>
       </c>
       <c r="C316" s="2" t="s">
         <v>904</v>
@@ -11499,15 +11499,15 @@
         <v>79</v>
       </c>
       <c r="E316" s="2" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
     </row>
     <row r="317" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A317" s="2" t="s">
+        <v>962</v>
+      </c>
+      <c r="B317" s="2" t="s">
         <v>963</v>
-      </c>
-      <c r="B317" s="2" t="s">
-        <v>964</v>
       </c>
       <c r="C317" s="2" t="s">
         <v>904</v>
@@ -11516,15 +11516,15 @@
         <v>122</v>
       </c>
       <c r="E317" s="2" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
     </row>
     <row r="318" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A318" s="2" t="s">
+        <v>965</v>
+      </c>
+      <c r="B318" s="2" t="s">
         <v>966</v>
-      </c>
-      <c r="B318" s="2" t="s">
-        <v>967</v>
       </c>
       <c r="C318" s="2" t="s">
         <v>904</v>
@@ -11533,15 +11533,15 @@
         <v>122</v>
       </c>
       <c r="E318" s="2" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
     </row>
     <row r="319" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A319" s="2" t="s">
+        <v>968</v>
+      </c>
+      <c r="B319" s="2" t="s">
         <v>969</v>
-      </c>
-      <c r="B319" s="2" t="s">
-        <v>970</v>
       </c>
       <c r="C319" s="2" t="s">
         <v>904</v>
@@ -11550,15 +11550,15 @@
         <v>122</v>
       </c>
       <c r="E319" s="2" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="320" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A320" s="2" t="s">
+        <v>971</v>
+      </c>
+      <c r="B320" s="2" t="s">
         <v>972</v>
-      </c>
-      <c r="B320" s="2" t="s">
-        <v>973</v>
       </c>
       <c r="C320" s="2" t="s">
         <v>904</v>
@@ -11567,15 +11567,15 @@
         <v>122</v>
       </c>
       <c r="E320" s="2" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
     </row>
     <row r="321" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A321" s="2" t="s">
+        <v>974</v>
+      </c>
+      <c r="B321" s="2" t="s">
         <v>975</v>
-      </c>
-      <c r="B321" s="2" t="s">
-        <v>976</v>
       </c>
       <c r="C321" s="2" t="s">
         <v>904</v>
@@ -11584,15 +11584,15 @@
         <v>122</v>
       </c>
       <c r="E321" s="2" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
     </row>
     <row r="322" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A322" s="2" t="s">
+        <v>977</v>
+      </c>
+      <c r="B322" s="2" t="s">
         <v>978</v>
-      </c>
-      <c r="B322" s="2" t="s">
-        <v>979</v>
       </c>
       <c r="C322" s="2" t="s">
         <v>904</v>
@@ -11601,15 +11601,15 @@
         <v>79</v>
       </c>
       <c r="E322" s="2" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
     </row>
     <row r="323" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A323" s="2" t="s">
+        <v>980</v>
+      </c>
+      <c r="B323" s="2" t="s">
         <v>981</v>
-      </c>
-      <c r="B323" s="2" t="s">
-        <v>982</v>
       </c>
       <c r="C323" s="2" t="s">
         <v>904</v>
@@ -11618,15 +11618,15 @@
         <v>27</v>
       </c>
       <c r="E323" s="2" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
     </row>
     <row r="324" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A324" s="2" t="s">
+        <v>983</v>
+      </c>
+      <c r="B324" s="2" t="s">
         <v>984</v>
-      </c>
-      <c r="B324" s="2" t="s">
-        <v>985</v>
       </c>
       <c r="C324" s="2" t="s">
         <v>904</v>
@@ -11635,15 +11635,15 @@
         <v>27</v>
       </c>
       <c r="E324" s="2" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
     </row>
     <row r="325" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A325" s="2" t="s">
+        <v>986</v>
+      </c>
+      <c r="B325" s="2" t="s">
         <v>987</v>
-      </c>
-      <c r="B325" s="2" t="s">
-        <v>988</v>
       </c>
       <c r="C325" s="2" t="s">
         <v>904</v>
@@ -11652,15 +11652,15 @@
         <v>122</v>
       </c>
       <c r="E325" s="2" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
     </row>
     <row r="326" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A326" s="2" t="s">
+        <v>989</v>
+      </c>
+      <c r="B326" s="2" t="s">
         <v>990</v>
-      </c>
-      <c r="B326" s="2" t="s">
-        <v>991</v>
       </c>
       <c r="C326" s="2" t="s">
         <v>904</v>
@@ -11669,3067 +11669,3067 @@
         <v>267</v>
       </c>
       <c r="E326" s="2" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
     </row>
     <row r="327" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A327" s="2" t="s">
+        <v>992</v>
+      </c>
+      <c r="B327" s="2" t="s">
         <v>993</v>
       </c>
-      <c r="B327" s="2" t="s">
+      <c r="C327" s="2" t="s">
         <v>994</v>
-      </c>
-      <c r="C327" s="2" t="s">
-        <v>995</v>
       </c>
       <c r="D327" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E327" s="2" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
     </row>
     <row r="328" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A328" s="2" t="s">
+        <v>996</v>
+      </c>
+      <c r="B328" s="2" t="s">
         <v>997</v>
       </c>
-      <c r="B328" s="2" t="s">
-        <v>998</v>
-      </c>
       <c r="C328" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D328" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E328" s="2" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
     </row>
     <row r="329" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A329" s="2" t="s">
+        <v>999</v>
+      </c>
+      <c r="B329" s="2" t="s">
         <v>1000</v>
       </c>
-      <c r="B329" s="2" t="s">
-        <v>1001</v>
-      </c>
       <c r="C329" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D329" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E329" s="2" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="330" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A330" s="2" t="s">
+        <v>1002</v>
+      </c>
+      <c r="B330" s="2" t="s">
         <v>1003</v>
       </c>
-      <c r="B330" s="2" t="s">
-        <v>1004</v>
-      </c>
       <c r="C330" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D330" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E330" s="2" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="331" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A331" s="2" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B331" s="2" t="s">
         <v>1006</v>
       </c>
-      <c r="B331" s="2" t="s">
-        <v>1007</v>
-      </c>
       <c r="C331" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D331" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E331" s="2" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="332" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A332" s="2" t="s">
+        <v>1008</v>
+      </c>
+      <c r="B332" s="2" t="s">
         <v>1009</v>
       </c>
-      <c r="B332" s="2" t="s">
-        <v>1010</v>
-      </c>
       <c r="C332" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D332" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E332" s="2" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="333" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A333" s="2" t="s">
+        <v>1011</v>
+      </c>
+      <c r="B333" s="2" t="s">
         <v>1012</v>
       </c>
-      <c r="B333" s="2" t="s">
-        <v>1013</v>
-      </c>
       <c r="C333" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D333" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E333" s="2" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="334" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A334" s="2" t="s">
+        <v>1014</v>
+      </c>
+      <c r="B334" s="2" t="s">
         <v>1015</v>
       </c>
-      <c r="B334" s="2" t="s">
-        <v>1016</v>
-      </c>
       <c r="C334" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D334" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E334" s="2" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="335" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A335" s="2" t="s">
+        <v>1017</v>
+      </c>
+      <c r="B335" s="2" t="s">
         <v>1018</v>
       </c>
-      <c r="B335" s="2" t="s">
-        <v>1019</v>
-      </c>
       <c r="C335" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D335" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E335" s="2" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="336" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A336" s="2" t="s">
+        <v>1020</v>
+      </c>
+      <c r="B336" s="2" t="s">
         <v>1021</v>
       </c>
-      <c r="B336" s="2" t="s">
-        <v>1022</v>
-      </c>
       <c r="C336" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D336" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E336" s="2" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="337" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A337" s="2" t="s">
+        <v>1023</v>
+      </c>
+      <c r="B337" s="2" t="s">
         <v>1024</v>
       </c>
-      <c r="B337" s="2" t="s">
-        <v>1025</v>
-      </c>
       <c r="C337" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D337" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E337" s="2" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="338" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A338" s="2" t="s">
+        <v>1026</v>
+      </c>
+      <c r="B338" s="2" t="s">
         <v>1027</v>
       </c>
-      <c r="B338" s="2" t="s">
-        <v>1028</v>
-      </c>
       <c r="C338" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D338" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E338" s="2" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="339" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A339" s="2" t="s">
+        <v>1029</v>
+      </c>
+      <c r="B339" s="2" t="s">
         <v>1030</v>
       </c>
-      <c r="B339" s="2" t="s">
-        <v>1031</v>
-      </c>
       <c r="C339" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D339" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E339" s="2" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="340" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A340" s="2" t="s">
+        <v>1032</v>
+      </c>
+      <c r="B340" s="2" t="s">
         <v>1033</v>
       </c>
-      <c r="B340" s="2" t="s">
-        <v>1034</v>
-      </c>
       <c r="C340" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D340" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E340" s="2" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
     </row>
     <row r="341" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A341" s="2" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B341" s="2" t="s">
         <v>1036</v>
       </c>
-      <c r="B341" s="2" t="s">
-        <v>1037</v>
-      </c>
       <c r="C341" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D341" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E341" s="2" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="342" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A342" s="2" t="s">
+        <v>1038</v>
+      </c>
+      <c r="B342" s="2" t="s">
         <v>1039</v>
       </c>
-      <c r="B342" s="2" t="s">
-        <v>1040</v>
-      </c>
       <c r="C342" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D342" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E342" s="2" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="343" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A343" s="2" t="s">
+        <v>1041</v>
+      </c>
+      <c r="B343" s="2" t="s">
         <v>1042</v>
       </c>
-      <c r="B343" s="2" t="s">
-        <v>1043</v>
-      </c>
       <c r="C343" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D343" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E343" s="2" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="344" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A344" s="2" t="s">
+        <v>1044</v>
+      </c>
+      <c r="B344" s="2" t="s">
         <v>1045</v>
       </c>
-      <c r="B344" s="2" t="s">
-        <v>1046</v>
-      </c>
       <c r="C344" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D344" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E344" s="2" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="345" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A345" s="2" t="s">
+        <v>1047</v>
+      </c>
+      <c r="B345" s="2" t="s">
         <v>1048</v>
       </c>
-      <c r="B345" s="2" t="s">
-        <v>1049</v>
-      </c>
       <c r="C345" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D345" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E345" s="2" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="346" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A346" s="2" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B346" s="2" t="s">
         <v>1051</v>
       </c>
-      <c r="B346" s="2" t="s">
-        <v>1052</v>
-      </c>
       <c r="C346" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D346" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E346" s="2" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="347" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A347" s="2" t="s">
+        <v>1053</v>
+      </c>
+      <c r="B347" s="2" t="s">
         <v>1054</v>
       </c>
-      <c r="B347" s="2" t="s">
-        <v>1055</v>
-      </c>
       <c r="C347" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D347" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E347" s="2" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="348" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A348" s="2" t="s">
+        <v>1056</v>
+      </c>
+      <c r="B348" s="2" t="s">
         <v>1057</v>
       </c>
-      <c r="B348" s="2" t="s">
-        <v>1058</v>
-      </c>
       <c r="C348" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D348" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E348" s="2" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="349" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A349" s="2" t="s">
+        <v>1059</v>
+      </c>
+      <c r="B349" s="2" t="s">
         <v>1060</v>
       </c>
-      <c r="B349" s="2" t="s">
-        <v>1061</v>
-      </c>
       <c r="C349" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D349" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E349" s="2" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="350" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A350" s="2" t="s">
+        <v>1062</v>
+      </c>
+      <c r="B350" s="2" t="s">
         <v>1063</v>
       </c>
-      <c r="B350" s="2" t="s">
-        <v>1064</v>
-      </c>
       <c r="C350" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D350" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E350" s="2" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="351" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A351" s="2" t="s">
+        <v>1065</v>
+      </c>
+      <c r="B351" s="2" t="s">
         <v>1066</v>
       </c>
-      <c r="B351" s="2" t="s">
-        <v>1067</v>
-      </c>
       <c r="C351" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D351" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E351" s="2" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="352" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A352" s="2" t="s">
+        <v>1068</v>
+      </c>
+      <c r="B352" s="2" t="s">
         <v>1069</v>
       </c>
-      <c r="B352" s="2" t="s">
-        <v>1070</v>
-      </c>
       <c r="C352" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D352" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E352" s="2" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="353" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A353" s="2" t="s">
+        <v>1071</v>
+      </c>
+      <c r="B353" s="2" t="s">
         <v>1072</v>
       </c>
-      <c r="B353" s="2" t="s">
-        <v>1073</v>
-      </c>
       <c r="C353" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D353" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E353" s="2" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="354" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A354" s="2" t="s">
+        <v>1074</v>
+      </c>
+      <c r="B354" s="2" t="s">
         <v>1075</v>
       </c>
-      <c r="B354" s="2" t="s">
-        <v>1076</v>
-      </c>
       <c r="C354" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D354" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E354" s="2" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="355" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A355" s="2" t="s">
+        <v>1077</v>
+      </c>
+      <c r="B355" s="2" t="s">
         <v>1078</v>
       </c>
-      <c r="B355" s="2" t="s">
-        <v>1079</v>
-      </c>
       <c r="C355" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D355" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E355" s="2" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="356" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A356" s="2" t="s">
+        <v>1080</v>
+      </c>
+      <c r="B356" s="2" t="s">
         <v>1081</v>
       </c>
-      <c r="B356" s="2" t="s">
-        <v>1082</v>
-      </c>
       <c r="C356" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D356" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E356" s="2" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="357" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A357" s="2" t="s">
+        <v>1083</v>
+      </c>
+      <c r="B357" s="2" t="s">
         <v>1084</v>
       </c>
-      <c r="B357" s="2" t="s">
+      <c r="C357" s="2" t="s">
         <v>1085</v>
-      </c>
-      <c r="C357" s="2" t="s">
-        <v>1086</v>
       </c>
       <c r="D357" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E357" s="2" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="358" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A358" s="2" t="s">
+        <v>1087</v>
+      </c>
+      <c r="B358" s="2" t="s">
         <v>1088</v>
       </c>
-      <c r="B358" s="2" t="s">
-        <v>1089</v>
-      </c>
       <c r="C358" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D358" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E358" s="2" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="359" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A359" s="2" t="s">
+        <v>1090</v>
+      </c>
+      <c r="B359" s="2" t="s">
         <v>1091</v>
       </c>
-      <c r="B359" s="2" t="s">
-        <v>1092</v>
-      </c>
       <c r="C359" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D359" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E359" s="2" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="360" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A360" s="2" t="s">
+        <v>1093</v>
+      </c>
+      <c r="B360" s="2" t="s">
         <v>1094</v>
       </c>
-      <c r="B360" s="2" t="s">
-        <v>1095</v>
-      </c>
       <c r="C360" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D360" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E360" s="2" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="361" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A361" s="2" t="s">
+        <v>1096</v>
+      </c>
+      <c r="B361" s="2" t="s">
         <v>1097</v>
       </c>
-      <c r="B361" s="2" t="s">
-        <v>1098</v>
-      </c>
       <c r="C361" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D361" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E361" s="2" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="362" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A362" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="B362" s="2" t="s">
         <v>1100</v>
       </c>
-      <c r="B362" s="2" t="s">
-        <v>1101</v>
-      </c>
       <c r="C362" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D362" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E362" s="2" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="363" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A363" s="2" t="s">
+        <v>1102</v>
+      </c>
+      <c r="B363" s="2" t="s">
         <v>1103</v>
       </c>
-      <c r="B363" s="2" t="s">
-        <v>1104</v>
-      </c>
       <c r="C363" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D363" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E363" s="2" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="364" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A364" s="2" t="s">
+        <v>1105</v>
+      </c>
+      <c r="B364" s="2" t="s">
         <v>1106</v>
       </c>
-      <c r="B364" s="2" t="s">
-        <v>1107</v>
-      </c>
       <c r="C364" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D364" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E364" s="2" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="365" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A365" s="2" t="s">
+        <v>1108</v>
+      </c>
+      <c r="B365" s="2" t="s">
         <v>1109</v>
       </c>
-      <c r="B365" s="2" t="s">
-        <v>1110</v>
-      </c>
       <c r="C365" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D365" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E365" s="2" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="366" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A366" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="B366" s="2" t="s">
         <v>1112</v>
       </c>
-      <c r="B366" s="2" t="s">
-        <v>1113</v>
-      </c>
       <c r="C366" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D366" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E366" s="2" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="367" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A367" s="2" t="s">
+        <v>1114</v>
+      </c>
+      <c r="B367" s="2" t="s">
         <v>1115</v>
       </c>
-      <c r="B367" s="2" t="s">
-        <v>1116</v>
-      </c>
       <c r="C367" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D367" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E367" s="2" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="368" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A368" s="2" t="s">
+        <v>1117</v>
+      </c>
+      <c r="B368" s="2" t="s">
         <v>1118</v>
       </c>
-      <c r="B368" s="2" t="s">
-        <v>1119</v>
-      </c>
       <c r="C368" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D368" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E368" s="2" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="369" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A369" s="2" t="s">
+        <v>1120</v>
+      </c>
+      <c r="B369" s="2" t="s">
         <v>1121</v>
       </c>
-      <c r="B369" s="2" t="s">
-        <v>1122</v>
-      </c>
       <c r="C369" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D369" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E369" s="2" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="370" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A370" s="2" t="s">
+        <v>1123</v>
+      </c>
+      <c r="B370" s="2" t="s">
         <v>1124</v>
       </c>
-      <c r="B370" s="2" t="s">
-        <v>1125</v>
-      </c>
       <c r="C370" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D370" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E370" s="2" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="371" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A371" s="2" t="s">
+        <v>1126</v>
+      </c>
+      <c r="B371" s="2" t="s">
         <v>1127</v>
       </c>
-      <c r="B371" s="2" t="s">
-        <v>1128</v>
-      </c>
       <c r="C371" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D371" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E371" s="2" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="372" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A372" s="2" t="s">
+        <v>1129</v>
+      </c>
+      <c r="B372" s="2" t="s">
         <v>1130</v>
       </c>
-      <c r="B372" s="2" t="s">
-        <v>1131</v>
-      </c>
       <c r="C372" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D372" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E372" s="2" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="373" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A373" s="2" t="s">
+        <v>1132</v>
+      </c>
+      <c r="B373" s="2" t="s">
         <v>1133</v>
       </c>
-      <c r="B373" s="2" t="s">
-        <v>1134</v>
-      </c>
       <c r="C373" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D373" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E373" s="2" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="374" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A374" s="2" t="s">
+        <v>1135</v>
+      </c>
+      <c r="B374" s="2" t="s">
         <v>1136</v>
       </c>
-      <c r="B374" s="2" t="s">
-        <v>1137</v>
-      </c>
       <c r="C374" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D374" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E374" s="2" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="375" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A375" s="2" t="s">
+        <v>1138</v>
+      </c>
+      <c r="B375" s="2" t="s">
         <v>1139</v>
       </c>
-      <c r="B375" s="2" t="s">
-        <v>1140</v>
-      </c>
       <c r="C375" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D375" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E375" s="2" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="376" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A376" s="2" t="s">
+        <v>1141</v>
+      </c>
+      <c r="B376" s="2" t="s">
         <v>1142</v>
       </c>
-      <c r="B376" s="2" t="s">
-        <v>1143</v>
-      </c>
       <c r="C376" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D376" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E376" s="2" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="377" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A377" s="2" t="s">
+        <v>1144</v>
+      </c>
+      <c r="B377" s="2" t="s">
         <v>1145</v>
       </c>
-      <c r="B377" s="2" t="s">
-        <v>1146</v>
-      </c>
       <c r="C377" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D377" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E377" s="2" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="378" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A378" s="2" t="s">
+        <v>1147</v>
+      </c>
+      <c r="B378" s="2" t="s">
         <v>1148</v>
       </c>
-      <c r="B378" s="2" t="s">
-        <v>1149</v>
-      </c>
       <c r="C378" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D378" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E378" s="2" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="379" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A379" s="2" t="s">
+        <v>1150</v>
+      </c>
+      <c r="B379" s="2" t="s">
         <v>1151</v>
       </c>
-      <c r="B379" s="2" t="s">
-        <v>1152</v>
-      </c>
       <c r="C379" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D379" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E379" s="2" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="380" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A380" s="2" t="s">
+        <v>1153</v>
+      </c>
+      <c r="B380" s="2" t="s">
         <v>1154</v>
       </c>
-      <c r="B380" s="2" t="s">
-        <v>1155</v>
-      </c>
       <c r="C380" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D380" s="2" t="s">
         <v>212</v>
       </c>
       <c r="E380" s="2" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="381" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A381" s="2" t="s">
+        <v>1156</v>
+      </c>
+      <c r="B381" s="2" t="s">
         <v>1157</v>
       </c>
-      <c r="B381" s="2" t="s">
-        <v>1158</v>
-      </c>
       <c r="C381" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D381" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E381" s="2" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="382" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A382" s="2" t="s">
+        <v>1159</v>
+      </c>
+      <c r="B382" s="2" t="s">
         <v>1160</v>
       </c>
-      <c r="B382" s="2" t="s">
-        <v>1161</v>
-      </c>
       <c r="C382" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D382" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E382" s="2" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="383" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A383" s="2" t="s">
+        <v>1162</v>
+      </c>
+      <c r="B383" s="2" t="s">
         <v>1163</v>
       </c>
-      <c r="B383" s="2" t="s">
-        <v>1164</v>
-      </c>
       <c r="C383" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D383" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E383" s="2" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="384" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A384" s="2" t="s">
+        <v>1165</v>
+      </c>
+      <c r="B384" s="2" t="s">
         <v>1166</v>
       </c>
-      <c r="B384" s="2" t="s">
-        <v>1167</v>
-      </c>
       <c r="C384" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D384" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E384" s="2" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="385" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A385" s="2" t="s">
+        <v>1168</v>
+      </c>
+      <c r="B385" s="2" t="s">
         <v>1169</v>
       </c>
-      <c r="B385" s="2" t="s">
-        <v>1170</v>
-      </c>
       <c r="C385" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D385" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E385" s="2" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="386" spans="1:5" s="2" customFormat="1" ht="135" x14ac:dyDescent="0.25">
       <c r="A386" s="2" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B386" s="2" t="s">
         <v>1172</v>
       </c>
-      <c r="B386" s="2" t="s">
-        <v>1173</v>
-      </c>
       <c r="C386" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D386" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E386" s="2" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="387" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A387" s="2" t="s">
+        <v>1174</v>
+      </c>
+      <c r="B387" s="2" t="s">
         <v>1175</v>
       </c>
-      <c r="B387" s="2" t="s">
+      <c r="C387" s="2" t="s">
         <v>1176</v>
-      </c>
-      <c r="C387" s="2" t="s">
-        <v>1177</v>
       </c>
       <c r="D387" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E387" s="2" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
     </row>
     <row r="388" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A388" s="2" t="s">
+        <v>1178</v>
+      </c>
+      <c r="B388" s="2" t="s">
         <v>1179</v>
       </c>
-      <c r="B388" s="2" t="s">
-        <v>1180</v>
-      </c>
       <c r="C388" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D388" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E388" s="2" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="389" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A389" s="2" t="s">
+        <v>1181</v>
+      </c>
+      <c r="B389" s="2" t="s">
         <v>1182</v>
       </c>
-      <c r="B389" s="2" t="s">
-        <v>1183</v>
-      </c>
       <c r="C389" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D389" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E389" s="2" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="390" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A390" s="2" t="s">
+        <v>1184</v>
+      </c>
+      <c r="B390" s="2" t="s">
         <v>1185</v>
       </c>
-      <c r="B390" s="2" t="s">
-        <v>1186</v>
-      </c>
       <c r="C390" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D390" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E390" s="2" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="391" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A391" s="2" t="s">
+        <v>1187</v>
+      </c>
+      <c r="B391" s="2" t="s">
         <v>1188</v>
       </c>
-      <c r="B391" s="2" t="s">
-        <v>1189</v>
-      </c>
       <c r="C391" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D391" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E391" s="2" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="392" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A392" s="2" t="s">
+        <v>1190</v>
+      </c>
+      <c r="B392" s="2" t="s">
         <v>1191</v>
       </c>
-      <c r="B392" s="2" t="s">
-        <v>1192</v>
-      </c>
       <c r="C392" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D392" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E392" s="2" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="393" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A393" s="2" t="s">
+        <v>1193</v>
+      </c>
+      <c r="B393" s="2" t="s">
         <v>1194</v>
       </c>
-      <c r="B393" s="2" t="s">
-        <v>1195</v>
-      </c>
       <c r="C393" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D393" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E393" s="2" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="394" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A394" s="2" t="s">
+        <v>1196</v>
+      </c>
+      <c r="B394" s="2" t="s">
         <v>1197</v>
       </c>
-      <c r="B394" s="2" t="s">
-        <v>1198</v>
-      </c>
       <c r="C394" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D394" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E394" s="2" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="395" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A395" s="2" t="s">
+        <v>1199</v>
+      </c>
+      <c r="B395" s="2" t="s">
         <v>1200</v>
       </c>
-      <c r="B395" s="2" t="s">
-        <v>1201</v>
-      </c>
       <c r="C395" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D395" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E395" s="2" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="396" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A396" s="2" t="s">
+        <v>1202</v>
+      </c>
+      <c r="B396" s="2" t="s">
         <v>1203</v>
       </c>
-      <c r="B396" s="2" t="s">
-        <v>1204</v>
-      </c>
       <c r="C396" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D396" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E396" s="2" t="s">
-        <v>1205</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="397" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A397" s="2" t="s">
+        <v>1205</v>
+      </c>
+      <c r="B397" s="2" t="s">
         <v>1206</v>
       </c>
-      <c r="B397" s="2" t="s">
-        <v>1207</v>
-      </c>
       <c r="C397" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D397" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E397" s="2" t="s">
-        <v>1208</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="398" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A398" s="2" t="s">
+        <v>1208</v>
+      </c>
+      <c r="B398" s="2" t="s">
         <v>1209</v>
       </c>
-      <c r="B398" s="2" t="s">
-        <v>1210</v>
-      </c>
       <c r="C398" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D398" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E398" s="2" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
     </row>
     <row r="399" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A399" s="2" t="s">
+        <v>1211</v>
+      </c>
+      <c r="B399" s="2" t="s">
         <v>1212</v>
       </c>
-      <c r="B399" s="2" t="s">
-        <v>1213</v>
-      </c>
       <c r="C399" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D399" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E399" s="2" t="s">
-        <v>1214</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="400" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A400" s="2" t="s">
+        <v>1214</v>
+      </c>
+      <c r="B400" s="2" t="s">
         <v>1215</v>
       </c>
-      <c r="B400" s="2" t="s">
-        <v>1216</v>
-      </c>
       <c r="C400" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D400" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E400" s="2" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="401" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A401" s="2" t="s">
+        <v>1217</v>
+      </c>
+      <c r="B401" s="2" t="s">
         <v>1218</v>
       </c>
-      <c r="B401" s="2" t="s">
-        <v>1219</v>
-      </c>
       <c r="C401" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D401" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E401" s="2" t="s">
-        <v>1220</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="402" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A402" s="2" t="s">
+        <v>1220</v>
+      </c>
+      <c r="B402" s="2" t="s">
         <v>1221</v>
       </c>
-      <c r="B402" s="2" t="s">
-        <v>1222</v>
-      </c>
       <c r="C402" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D402" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E402" s="2" t="s">
-        <v>1223</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="403" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A403" s="2" t="s">
+        <v>1223</v>
+      </c>
+      <c r="B403" s="2" t="s">
         <v>1224</v>
       </c>
-      <c r="B403" s="2" t="s">
-        <v>1225</v>
-      </c>
       <c r="C403" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D403" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E403" s="2" t="s">
-        <v>1226</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="404" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A404" s="2" t="s">
+        <v>1226</v>
+      </c>
+      <c r="B404" s="2" t="s">
         <v>1227</v>
       </c>
-      <c r="B404" s="2" t="s">
-        <v>1228</v>
-      </c>
       <c r="C404" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D404" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E404" s="2" t="s">
-        <v>1229</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="405" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A405" s="2" t="s">
+        <v>1229</v>
+      </c>
+      <c r="B405" s="2" t="s">
         <v>1230</v>
       </c>
-      <c r="B405" s="2" t="s">
-        <v>1231</v>
-      </c>
       <c r="C405" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D405" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E405" s="2" t="s">
-        <v>1232</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="406" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A406" s="2" t="s">
+        <v>1232</v>
+      </c>
+      <c r="B406" s="2" t="s">
         <v>1233</v>
       </c>
-      <c r="B406" s="2" t="s">
-        <v>1234</v>
-      </c>
       <c r="C406" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D406" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E406" s="2" t="s">
-        <v>1235</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="407" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A407" s="2" t="s">
+        <v>1235</v>
+      </c>
+      <c r="B407" s="2" t="s">
         <v>1236</v>
       </c>
-      <c r="B407" s="2" t="s">
-        <v>1237</v>
-      </c>
       <c r="C407" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D407" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E407" s="2" t="s">
-        <v>1238</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="408" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A408" s="2" t="s">
-        <v>1239</v>
+        <v>1238</v>
       </c>
       <c r="B408" s="2" t="s">
         <v>715</v>
       </c>
       <c r="C408" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D408" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E408" s="2" t="s">
-        <v>1240</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="409" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A409" s="2" t="s">
+        <v>1240</v>
+      </c>
+      <c r="B409" s="2" t="s">
         <v>1241</v>
       </c>
-      <c r="B409" s="2" t="s">
-        <v>1242</v>
-      </c>
       <c r="C409" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D409" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E409" s="2" t="s">
-        <v>1243</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="410" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A410" s="2" t="s">
+        <v>1243</v>
+      </c>
+      <c r="B410" s="2" t="s">
         <v>1244</v>
       </c>
-      <c r="B410" s="2" t="s">
-        <v>1245</v>
-      </c>
       <c r="C410" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D410" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E410" s="2" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="411" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A411" s="2" t="s">
+        <v>1246</v>
+      </c>
+      <c r="B411" s="2" t="s">
         <v>1247</v>
       </c>
-      <c r="B411" s="2" t="s">
-        <v>1248</v>
-      </c>
       <c r="C411" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D411" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E411" s="2" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
     </row>
     <row r="412" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A412" s="2" t="s">
+        <v>1249</v>
+      </c>
+      <c r="B412" s="2" t="s">
         <v>1250</v>
       </c>
-      <c r="B412" s="2" t="s">
-        <v>1251</v>
-      </c>
       <c r="C412" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D412" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E412" s="2" t="s">
-        <v>1252</v>
+        <v>1251</v>
       </c>
     </row>
     <row r="413" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A413" s="2" t="s">
+        <v>1252</v>
+      </c>
+      <c r="B413" s="2" t="s">
         <v>1253</v>
       </c>
-      <c r="B413" s="2" t="s">
-        <v>1254</v>
-      </c>
       <c r="C413" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D413" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E413" s="2" t="s">
-        <v>1255</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="414" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A414" s="2" t="s">
+        <v>1255</v>
+      </c>
+      <c r="B414" s="2" t="s">
         <v>1256</v>
       </c>
-      <c r="B414" s="2" t="s">
-        <v>1257</v>
-      </c>
       <c r="C414" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D414" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E414" s="2" t="s">
-        <v>1258</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="415" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A415" s="2" t="s">
+        <v>1258</v>
+      </c>
+      <c r="B415" s="2" t="s">
         <v>1259</v>
       </c>
-      <c r="B415" s="2" t="s">
-        <v>1260</v>
-      </c>
       <c r="C415" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D415" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E415" s="2" t="s">
-        <v>1261</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="416" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A416" s="2" t="s">
+        <v>1261</v>
+      </c>
+      <c r="B416" s="2" t="s">
         <v>1262</v>
       </c>
-      <c r="B416" s="2" t="s">
-        <v>1263</v>
-      </c>
       <c r="C416" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D416" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E416" s="2" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
     </row>
     <row r="417" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A417" s="2" t="s">
+        <v>1264</v>
+      </c>
+      <c r="B417" s="2" t="s">
         <v>1265</v>
       </c>
-      <c r="B417" s="2" t="s">
+      <c r="C417" s="2" t="s">
         <v>1266</v>
-      </c>
-      <c r="C417" s="2" t="s">
-        <v>1267</v>
       </c>
       <c r="D417" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E417" s="2" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="418" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A418" s="2" t="s">
+        <v>1268</v>
+      </c>
+      <c r="B418" s="2" t="s">
         <v>1269</v>
       </c>
-      <c r="B418" s="2" t="s">
-        <v>1270</v>
-      </c>
       <c r="C418" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D418" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E418" s="2" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="419" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A419" s="2" t="s">
+        <v>1271</v>
+      </c>
+      <c r="B419" s="2" t="s">
         <v>1272</v>
       </c>
-      <c r="B419" s="2" t="s">
-        <v>1273</v>
-      </c>
       <c r="C419" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D419" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E419" s="2" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="420" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A420" s="2" t="s">
+        <v>1274</v>
+      </c>
+      <c r="B420" s="2" t="s">
         <v>1275</v>
       </c>
-      <c r="B420" s="2" t="s">
-        <v>1276</v>
-      </c>
       <c r="C420" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D420" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E420" s="2" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="421" spans="1:5" s="2" customFormat="1" ht="105" x14ac:dyDescent="0.25">
       <c r="A421" s="2" t="s">
+        <v>1277</v>
+      </c>
+      <c r="B421" s="2" t="s">
         <v>1278</v>
       </c>
-      <c r="B421" s="2" t="s">
-        <v>1279</v>
-      </c>
       <c r="C421" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D421" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E421" s="2" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="422" spans="1:5" s="2" customFormat="1" ht="105" x14ac:dyDescent="0.25">
       <c r="A422" s="2" t="s">
+        <v>1280</v>
+      </c>
+      <c r="B422" s="2" t="s">
         <v>1281</v>
       </c>
-      <c r="B422" s="2" t="s">
-        <v>1282</v>
-      </c>
       <c r="C422" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D422" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E422" s="2" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
     </row>
     <row r="423" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A423" s="2" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B423" s="2" t="s">
         <v>1284</v>
       </c>
-      <c r="B423" s="2" t="s">
-        <v>1285</v>
-      </c>
       <c r="C423" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D423" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E423" s="2" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="424" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A424" s="2" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B424" s="2" t="s">
         <v>1287</v>
       </c>
-      <c r="B424" s="2" t="s">
-        <v>1288</v>
-      </c>
       <c r="C424" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D424" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E424" s="2" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="425" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A425" s="2" t="s">
+        <v>1289</v>
+      </c>
+      <c r="B425" s="2" t="s">
         <v>1290</v>
       </c>
-      <c r="B425" s="2" t="s">
-        <v>1291</v>
-      </c>
       <c r="C425" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D425" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E425" s="2" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
     </row>
     <row r="426" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A426" s="2" t="s">
+        <v>1292</v>
+      </c>
+      <c r="B426" s="2" t="s">
         <v>1293</v>
       </c>
-      <c r="B426" s="2" t="s">
-        <v>1294</v>
-      </c>
       <c r="C426" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D426" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E426" s="2" t="s">
-        <v>1295</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="427" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A427" s="2" t="s">
+        <v>1295</v>
+      </c>
+      <c r="B427" s="2" t="s">
         <v>1296</v>
       </c>
-      <c r="B427" s="2" t="s">
-        <v>1297</v>
-      </c>
       <c r="C427" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D427" s="2" t="s">
         <v>212</v>
       </c>
       <c r="E427" s="2" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="428" spans="1:5" s="2" customFormat="1" ht="105" x14ac:dyDescent="0.25">
       <c r="A428" s="2" t="s">
+        <v>1298</v>
+      </c>
+      <c r="B428" s="2" t="s">
         <v>1299</v>
       </c>
-      <c r="B428" s="2" t="s">
-        <v>1300</v>
-      </c>
       <c r="C428" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D428" s="2" t="s">
         <v>212</v>
       </c>
       <c r="E428" s="2" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="429" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A429" s="2" t="s">
+        <v>1301</v>
+      </c>
+      <c r="B429" s="2" t="s">
         <v>1302</v>
       </c>
-      <c r="B429" s="2" t="s">
-        <v>1303</v>
-      </c>
       <c r="C429" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D429" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E429" s="2" t="s">
-        <v>1304</v>
+        <v>1303</v>
       </c>
     </row>
     <row r="430" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A430" s="2" t="s">
+        <v>1304</v>
+      </c>
+      <c r="B430" s="2" t="s">
         <v>1305</v>
       </c>
-      <c r="B430" s="2" t="s">
-        <v>1306</v>
-      </c>
       <c r="C430" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D430" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E430" s="2" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
     </row>
     <row r="431" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A431" s="2" t="s">
+        <v>1307</v>
+      </c>
+      <c r="B431" s="2" t="s">
         <v>1308</v>
       </c>
-      <c r="B431" s="2" t="s">
-        <v>1309</v>
-      </c>
       <c r="C431" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D431" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E431" s="2" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="432" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A432" s="2" t="s">
+        <v>1310</v>
+      </c>
+      <c r="B432" s="2" t="s">
         <v>1311</v>
       </c>
-      <c r="B432" s="2" t="s">
-        <v>1312</v>
-      </c>
       <c r="C432" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D432" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E432" s="2" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="433" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A433" s="2" t="s">
+        <v>1313</v>
+      </c>
+      <c r="B433" s="2" t="s">
         <v>1314</v>
       </c>
-      <c r="B433" s="2" t="s">
-        <v>1315</v>
-      </c>
       <c r="C433" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D433" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E433" s="2" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="434" spans="1:5" s="2" customFormat="1" ht="105" x14ac:dyDescent="0.25">
       <c r="A434" s="2" t="s">
+        <v>1316</v>
+      </c>
+      <c r="B434" s="2" t="s">
         <v>1317</v>
       </c>
-      <c r="B434" s="2" t="s">
-        <v>1318</v>
-      </c>
       <c r="C434" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D434" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E434" s="2" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="435" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A435" s="2" t="s">
+        <v>1319</v>
+      </c>
+      <c r="B435" s="2" t="s">
         <v>1320</v>
       </c>
-      <c r="B435" s="2" t="s">
-        <v>1321</v>
-      </c>
       <c r="C435" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D435" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E435" s="2" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="436" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A436" s="2" t="s">
+        <v>1322</v>
+      </c>
+      <c r="B436" s="2" t="s">
         <v>1323</v>
       </c>
-      <c r="B436" s="2" t="s">
-        <v>1324</v>
-      </c>
       <c r="C436" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D436" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E436" s="2" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="437" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A437" s="2" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B437" s="2" t="s">
         <v>1326</v>
       </c>
-      <c r="B437" s="2" t="s">
-        <v>1327</v>
-      </c>
       <c r="C437" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D437" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E437" s="2" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
     </row>
     <row r="438" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A438" s="2" t="s">
+        <v>1328</v>
+      </c>
+      <c r="B438" s="2" t="s">
         <v>1329</v>
       </c>
-      <c r="B438" s="2" t="s">
-        <v>1330</v>
-      </c>
       <c r="C438" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D438" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E438" s="2" t="s">
-        <v>1331</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="439" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A439" s="2" t="s">
+        <v>1331</v>
+      </c>
+      <c r="B439" s="2" t="s">
         <v>1332</v>
       </c>
-      <c r="B439" s="2" t="s">
-        <v>1333</v>
-      </c>
       <c r="C439" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D439" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E439" s="2" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="440" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A440" s="2" t="s">
+        <v>1334</v>
+      </c>
+      <c r="B440" s="2" t="s">
         <v>1335</v>
       </c>
-      <c r="B440" s="2" t="s">
-        <v>1336</v>
-      </c>
       <c r="C440" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D440" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E440" s="2" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="441" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A441" s="2" t="s">
+        <v>1337</v>
+      </c>
+      <c r="B441" s="2" t="s">
         <v>1338</v>
       </c>
-      <c r="B441" s="2" t="s">
-        <v>1339</v>
-      </c>
       <c r="C441" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D441" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E441" s="2" t="s">
-        <v>1340</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="442" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A442" s="2" t="s">
+        <v>1340</v>
+      </c>
+      <c r="B442" s="2" t="s">
         <v>1341</v>
       </c>
-      <c r="B442" s="2" t="s">
-        <v>1342</v>
-      </c>
       <c r="C442" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D442" s="2" t="s">
         <v>212</v>
       </c>
       <c r="E442" s="2" t="s">
-        <v>1343</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="443" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A443" s="2" t="s">
+        <v>1343</v>
+      </c>
+      <c r="B443" s="2" t="s">
         <v>1344</v>
       </c>
-      <c r="B443" s="2" t="s">
-        <v>1345</v>
-      </c>
       <c r="C443" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D443" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E443" s="2" t="s">
-        <v>1346</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="444" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A444" s="2" t="s">
+        <v>1346</v>
+      </c>
+      <c r="B444" s="2" t="s">
         <v>1347</v>
       </c>
-      <c r="B444" s="2" t="s">
-        <v>1348</v>
-      </c>
       <c r="C444" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D444" s="2" t="s">
         <v>212</v>
       </c>
       <c r="E444" s="2" t="s">
-        <v>1349</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="445" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A445" s="2" t="s">
+        <v>1349</v>
+      </c>
+      <c r="B445" s="2" t="s">
         <v>1350</v>
       </c>
-      <c r="B445" s="2" t="s">
-        <v>1351</v>
-      </c>
       <c r="C445" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D445" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E445" s="2" t="s">
-        <v>1352</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="446" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A446" s="2" t="s">
+        <v>1352</v>
+      </c>
+      <c r="B446" s="2" t="s">
         <v>1353</v>
       </c>
-      <c r="B446" s="2" t="s">
-        <v>1354</v>
-      </c>
       <c r="C446" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D446" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E446" s="2" t="s">
-        <v>1355</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="447" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A447" s="2" t="s">
+        <v>1355</v>
+      </c>
+      <c r="B447" s="2" t="s">
         <v>1356</v>
       </c>
-      <c r="B447" s="2" t="s">
+      <c r="C447" s="2" t="s">
         <v>1357</v>
-      </c>
-      <c r="C447" s="2" t="s">
-        <v>1358</v>
       </c>
       <c r="D447" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E447" s="2" t="s">
-        <v>1359</v>
+        <v>1358</v>
       </c>
     </row>
     <row r="448" spans="1:5" s="2" customFormat="1" ht="135" x14ac:dyDescent="0.25">
       <c r="A448" s="2" t="s">
+        <v>1359</v>
+      </c>
+      <c r="B448" s="2" t="s">
         <v>1360</v>
       </c>
-      <c r="B448" s="2" t="s">
-        <v>1361</v>
-      </c>
       <c r="C448" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D448" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E448" s="2" t="s">
-        <v>1362</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="449" spans="1:5" s="2" customFormat="1" ht="135" x14ac:dyDescent="0.25">
       <c r="A449" s="2" t="s">
+        <v>1362</v>
+      </c>
+      <c r="B449" s="2" t="s">
         <v>1363</v>
       </c>
-      <c r="B449" s="2" t="s">
-        <v>1364</v>
-      </c>
       <c r="C449" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D449" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E449" s="2" t="s">
-        <v>1365</v>
+        <v>1364</v>
       </c>
     </row>
     <row r="450" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A450" s="2" t="s">
+        <v>1365</v>
+      </c>
+      <c r="B450" s="2" t="s">
         <v>1366</v>
       </c>
-      <c r="B450" s="2" t="s">
-        <v>1367</v>
-      </c>
       <c r="C450" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D450" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E450" s="2" t="s">
-        <v>1368</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="451" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A451" s="2" t="s">
+        <v>1368</v>
+      </c>
+      <c r="B451" s="2" t="s">
         <v>1369</v>
       </c>
-      <c r="B451" s="2" t="s">
-        <v>1370</v>
-      </c>
       <c r="C451" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D451" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E451" s="2" t="s">
-        <v>1371</v>
+        <v>1370</v>
       </c>
     </row>
     <row r="452" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A452" s="2" t="s">
+        <v>1371</v>
+      </c>
+      <c r="B452" s="2" t="s">
         <v>1372</v>
       </c>
-      <c r="B452" s="2" t="s">
-        <v>1373</v>
-      </c>
       <c r="C452" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D452" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E452" s="2" t="s">
-        <v>1374</v>
+        <v>1373</v>
       </c>
     </row>
     <row r="453" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A453" s="2" t="s">
+        <v>1374</v>
+      </c>
+      <c r="B453" s="2" t="s">
         <v>1375</v>
       </c>
-      <c r="B453" s="2" t="s">
-        <v>1376</v>
-      </c>
       <c r="C453" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D453" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E453" s="2" t="s">
-        <v>1377</v>
+        <v>1376</v>
       </c>
     </row>
     <row r="454" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A454" s="2" t="s">
+        <v>1377</v>
+      </c>
+      <c r="B454" s="2" t="s">
         <v>1378</v>
       </c>
-      <c r="B454" s="2" t="s">
-        <v>1379</v>
-      </c>
       <c r="C454" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D454" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E454" s="2" t="s">
-        <v>1380</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="455" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A455" s="2" t="s">
+        <v>1380</v>
+      </c>
+      <c r="B455" s="2" t="s">
         <v>1381</v>
       </c>
-      <c r="B455" s="2" t="s">
-        <v>1382</v>
-      </c>
       <c r="C455" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D455" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E455" s="2" t="s">
-        <v>1383</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="456" spans="1:5" s="2" customFormat="1" ht="135" x14ac:dyDescent="0.25">
       <c r="A456" s="2" t="s">
+        <v>1383</v>
+      </c>
+      <c r="B456" s="2" t="s">
         <v>1384</v>
       </c>
-      <c r="B456" s="2" t="s">
-        <v>1385</v>
-      </c>
       <c r="C456" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D456" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E456" s="2" t="s">
-        <v>1386</v>
+        <v>1385</v>
       </c>
     </row>
     <row r="457" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A457" s="2" t="s">
+        <v>1386</v>
+      </c>
+      <c r="B457" s="2" t="s">
         <v>1387</v>
       </c>
-      <c r="B457" s="2" t="s">
-        <v>1388</v>
-      </c>
       <c r="C457" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D457" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E457" s="2" t="s">
-        <v>1389</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="458" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A458" s="2" t="s">
+        <v>1389</v>
+      </c>
+      <c r="B458" s="2" t="s">
         <v>1390</v>
       </c>
-      <c r="B458" s="2" t="s">
-        <v>1391</v>
-      </c>
       <c r="C458" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D458" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E458" s="2" t="s">
-        <v>1392</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="459" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A459" s="2" t="s">
+        <v>1392</v>
+      </c>
+      <c r="B459" s="2" t="s">
         <v>1393</v>
       </c>
-      <c r="B459" s="2" t="s">
-        <v>1394</v>
-      </c>
       <c r="C459" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D459" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E459" s="2" t="s">
-        <v>1395</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="460" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A460" s="2" t="s">
+        <v>1395</v>
+      </c>
+      <c r="B460" s="2" t="s">
         <v>1396</v>
       </c>
-      <c r="B460" s="2" t="s">
-        <v>1397</v>
-      </c>
       <c r="C460" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D460" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E460" s="2" t="s">
-        <v>1398</v>
+        <v>1397</v>
       </c>
     </row>
     <row r="461" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A461" s="2" t="s">
+        <v>1398</v>
+      </c>
+      <c r="B461" s="2" t="s">
         <v>1399</v>
       </c>
-      <c r="B461" s="2" t="s">
-        <v>1400</v>
-      </c>
       <c r="C461" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D461" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E461" s="2" t="s">
-        <v>1401</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="462" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A462" s="2" t="s">
+        <v>1401</v>
+      </c>
+      <c r="B462" s="2" t="s">
         <v>1402</v>
       </c>
-      <c r="B462" s="2" t="s">
-        <v>1403</v>
-      </c>
       <c r="C462" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D462" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E462" s="2" t="s">
-        <v>1404</v>
+        <v>1403</v>
       </c>
     </row>
     <row r="463" spans="1:5" s="2" customFormat="1" ht="135" x14ac:dyDescent="0.25">
       <c r="A463" s="2" t="s">
+        <v>1404</v>
+      </c>
+      <c r="B463" s="2" t="s">
         <v>1405</v>
       </c>
-      <c r="B463" s="2" t="s">
-        <v>1406</v>
-      </c>
       <c r="C463" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D463" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E463" s="2" t="s">
-        <v>1407</v>
+        <v>1406</v>
       </c>
     </row>
     <row r="464" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A464" s="2" t="s">
+        <v>1407</v>
+      </c>
+      <c r="B464" s="2" t="s">
         <v>1408</v>
       </c>
-      <c r="B464" s="2" t="s">
-        <v>1409</v>
-      </c>
       <c r="C464" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D464" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E464" s="2" t="s">
-        <v>1410</v>
+        <v>1409</v>
       </c>
     </row>
     <row r="465" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A465" s="2" t="s">
+        <v>1410</v>
+      </c>
+      <c r="B465" s="2" t="s">
         <v>1411</v>
       </c>
-      <c r="B465" s="2" t="s">
-        <v>1412</v>
-      </c>
       <c r="C465" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D465" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E465" s="2" t="s">
-        <v>1413</v>
+        <v>1412</v>
       </c>
     </row>
     <row r="466" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A466" s="2" t="s">
+        <v>1413</v>
+      </c>
+      <c r="B466" s="2" t="s">
         <v>1414</v>
       </c>
-      <c r="B466" s="2" t="s">
-        <v>1415</v>
-      </c>
       <c r="C466" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D466" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E466" s="2" t="s">
-        <v>1416</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="467" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A467" s="2" t="s">
+        <v>1416</v>
+      </c>
+      <c r="B467" s="2" t="s">
         <v>1417</v>
       </c>
-      <c r="B467" s="2" t="s">
-        <v>1418</v>
-      </c>
       <c r="C467" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D467" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E467" s="2" t="s">
-        <v>1419</v>
+        <v>1418</v>
       </c>
     </row>
     <row r="468" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A468" s="2" t="s">
+        <v>1419</v>
+      </c>
+      <c r="B468" s="2" t="s">
         <v>1420</v>
       </c>
-      <c r="B468" s="2" t="s">
-        <v>1421</v>
-      </c>
       <c r="C468" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D468" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E468" s="2" t="s">
-        <v>1422</v>
+        <v>1421</v>
       </c>
     </row>
     <row r="469" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A469" s="2" t="s">
+        <v>1422</v>
+      </c>
+      <c r="B469" s="2" t="s">
         <v>1423</v>
       </c>
-      <c r="B469" s="2" t="s">
-        <v>1424</v>
-      </c>
       <c r="C469" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D469" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E469" s="2" t="s">
-        <v>1425</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="470" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A470" s="2" t="s">
+        <v>1425</v>
+      </c>
+      <c r="B470" s="2" t="s">
         <v>1426</v>
       </c>
-      <c r="B470" s="2" t="s">
-        <v>1427</v>
-      </c>
       <c r="C470" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D470" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E470" s="2" t="s">
-        <v>1428</v>
+        <v>1427</v>
       </c>
     </row>
     <row r="471" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A471" s="2" t="s">
+        <v>1428</v>
+      </c>
+      <c r="B471" s="2" t="s">
         <v>1429</v>
       </c>
-      <c r="B471" s="2" t="s">
-        <v>1430</v>
-      </c>
       <c r="C471" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D471" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E471" s="2" t="s">
-        <v>1431</v>
+        <v>1430</v>
       </c>
     </row>
     <row r="472" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A472" s="2" t="s">
+        <v>1431</v>
+      </c>
+      <c r="B472" s="2" t="s">
         <v>1432</v>
       </c>
-      <c r="B472" s="2" t="s">
-        <v>1433</v>
-      </c>
       <c r="C472" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D472" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E472" s="2" t="s">
-        <v>1434</v>
+        <v>1433</v>
       </c>
     </row>
     <row r="473" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A473" s="2" t="s">
+        <v>1434</v>
+      </c>
+      <c r="B473" s="2" t="s">
         <v>1435</v>
       </c>
-      <c r="B473" s="2" t="s">
-        <v>1436</v>
-      </c>
       <c r="C473" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D473" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E473" s="2" t="s">
-        <v>1437</v>
+        <v>1436</v>
       </c>
     </row>
     <row r="474" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A474" s="2" t="s">
+        <v>1437</v>
+      </c>
+      <c r="B474" s="2" t="s">
         <v>1438</v>
       </c>
-      <c r="B474" s="2" t="s">
-        <v>1439</v>
-      </c>
       <c r="C474" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D474" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E474" s="2" t="s">
-        <v>1440</v>
+        <v>1439</v>
       </c>
     </row>
     <row r="475" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A475" s="2" t="s">
+        <v>1440</v>
+      </c>
+      <c r="B475" s="2" t="s">
         <v>1441</v>
       </c>
-      <c r="B475" s="2" t="s">
-        <v>1442</v>
-      </c>
       <c r="C475" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D475" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E475" s="2" t="s">
-        <v>1443</v>
+        <v>1442</v>
       </c>
     </row>
     <row r="476" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A476" s="2" t="s">
+        <v>1443</v>
+      </c>
+      <c r="B476" s="2" t="s">
         <v>1444</v>
       </c>
-      <c r="B476" s="2" t="s">
-        <v>1445</v>
-      </c>
       <c r="C476" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="D476" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E476" s="2" t="s">
-        <v>1446</v>
+        <v>1445</v>
       </c>
     </row>
     <row r="477" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A477" s="2" t="s">
+        <v>1446</v>
+      </c>
+      <c r="B477" s="2" t="s">
         <v>1447</v>
       </c>
-      <c r="B477" s="2" t="s">
+      <c r="C477" s="2" t="s">
         <v>1448</v>
-      </c>
-      <c r="C477" s="2" t="s">
-        <v>1449</v>
       </c>
       <c r="D477" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E477" s="2" t="s">
-        <v>1450</v>
+        <v>1449</v>
       </c>
     </row>
     <row r="478" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A478" s="2" t="s">
+        <v>1450</v>
+      </c>
+      <c r="B478" s="2" t="s">
         <v>1451</v>
       </c>
-      <c r="B478" s="2" t="s">
-        <v>1452</v>
-      </c>
       <c r="C478" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D478" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E478" s="2" t="s">
-        <v>1453</v>
+        <v>1452</v>
       </c>
     </row>
     <row r="479" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A479" s="2" t="s">
+        <v>1453</v>
+      </c>
+      <c r="B479" s="2" t="s">
         <v>1454</v>
       </c>
-      <c r="B479" s="2" t="s">
-        <v>1455</v>
-      </c>
       <c r="C479" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D479" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E479" s="2" t="s">
-        <v>1456</v>
+        <v>1455</v>
       </c>
     </row>
     <row r="480" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A480" s="2" t="s">
+        <v>1456</v>
+      </c>
+      <c r="B480" s="2" t="s">
         <v>1457</v>
       </c>
-      <c r="B480" s="2" t="s">
-        <v>1458</v>
-      </c>
       <c r="C480" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D480" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E480" s="2" t="s">
-        <v>1459</v>
+        <v>1458</v>
       </c>
     </row>
     <row r="481" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A481" s="2" t="s">
+        <v>1459</v>
+      </c>
+      <c r="B481" s="2" t="s">
         <v>1460</v>
       </c>
-      <c r="B481" s="2" t="s">
-        <v>1461</v>
-      </c>
       <c r="C481" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D481" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E481" s="2" t="s">
-        <v>1462</v>
+        <v>1461</v>
       </c>
     </row>
     <row r="482" spans="1:5" s="2" customFormat="1" ht="135" x14ac:dyDescent="0.25">
       <c r="A482" s="2" t="s">
+        <v>1462</v>
+      </c>
+      <c r="B482" s="2" t="s">
         <v>1463</v>
       </c>
-      <c r="B482" s="2" t="s">
-        <v>1464</v>
-      </c>
       <c r="C482" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D482" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E482" s="2" t="s">
-        <v>1465</v>
+        <v>1464</v>
       </c>
     </row>
     <row r="483" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A483" s="2" t="s">
+        <v>1465</v>
+      </c>
+      <c r="B483" s="2" t="s">
         <v>1466</v>
       </c>
-      <c r="B483" s="2" t="s">
-        <v>1467</v>
-      </c>
       <c r="C483" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D483" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E483" s="2" t="s">
-        <v>1468</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="484" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A484" s="2" t="s">
+        <v>1468</v>
+      </c>
+      <c r="B484" s="2" t="s">
         <v>1469</v>
       </c>
-      <c r="B484" s="2" t="s">
-        <v>1470</v>
-      </c>
       <c r="C484" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D484" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E484" s="2" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
     </row>
     <row r="485" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A485" s="2" t="s">
+        <v>1471</v>
+      </c>
+      <c r="B485" s="2" t="s">
         <v>1472</v>
       </c>
-      <c r="B485" s="2" t="s">
-        <v>1473</v>
-      </c>
       <c r="C485" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D485" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E485" s="2" t="s">
-        <v>1474</v>
+        <v>1473</v>
       </c>
     </row>
     <row r="486" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A486" s="2" t="s">
+        <v>1474</v>
+      </c>
+      <c r="B486" s="2" t="s">
         <v>1475</v>
       </c>
-      <c r="B486" s="2" t="s">
-        <v>1476</v>
-      </c>
       <c r="C486" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D486" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E486" s="2" t="s">
-        <v>1477</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="487" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A487" s="2" t="s">
+        <v>1477</v>
+      </c>
+      <c r="B487" s="2" t="s">
         <v>1478</v>
       </c>
-      <c r="B487" s="2" t="s">
-        <v>1479</v>
-      </c>
       <c r="C487" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D487" s="2" t="s">
         <v>79</v>
       </c>
       <c r="E487" s="2" t="s">
-        <v>1480</v>
+        <v>1479</v>
       </c>
     </row>
     <row r="488" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A488" s="2" t="s">
+        <v>1480</v>
+      </c>
+      <c r="B488" s="2" t="s">
         <v>1481</v>
       </c>
-      <c r="B488" s="2" t="s">
-        <v>1482</v>
-      </c>
       <c r="C488" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D488" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E488" s="2" t="s">
-        <v>1483</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="489" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A489" s="2" t="s">
+        <v>1483</v>
+      </c>
+      <c r="B489" s="2" t="s">
         <v>1484</v>
       </c>
-      <c r="B489" s="2" t="s">
-        <v>1485</v>
-      </c>
       <c r="C489" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D489" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E489" s="2" t="s">
-        <v>1486</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="490" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A490" s="2" t="s">
+        <v>1486</v>
+      </c>
+      <c r="B490" s="2" t="s">
         <v>1487</v>
       </c>
-      <c r="B490" s="2" t="s">
-        <v>1488</v>
-      </c>
       <c r="C490" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D490" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E490" s="2" t="s">
-        <v>1489</v>
+        <v>1488</v>
       </c>
     </row>
     <row r="491" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A491" s="2" t="s">
+        <v>1489</v>
+      </c>
+      <c r="B491" s="2" t="s">
         <v>1490</v>
       </c>
-      <c r="B491" s="2" t="s">
-        <v>1491</v>
-      </c>
       <c r="C491" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D491" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E491" s="2" t="s">
-        <v>1492</v>
+        <v>1491</v>
       </c>
     </row>
     <row r="492" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A492" s="2" t="s">
+        <v>1492</v>
+      </c>
+      <c r="B492" s="2" t="s">
         <v>1493</v>
       </c>
-      <c r="B492" s="2" t="s">
-        <v>1494</v>
-      </c>
       <c r="C492" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D492" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E492" s="2" t="s">
-        <v>1495</v>
+        <v>1494</v>
       </c>
     </row>
     <row r="493" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A493" s="2" t="s">
+        <v>1495</v>
+      </c>
+      <c r="B493" s="2" t="s">
         <v>1496</v>
       </c>
-      <c r="B493" s="2" t="s">
-        <v>1497</v>
-      </c>
       <c r="C493" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D493" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E493" s="2" t="s">
-        <v>1498</v>
+        <v>1497</v>
       </c>
     </row>
     <row r="494" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A494" s="2" t="s">
+        <v>1498</v>
+      </c>
+      <c r="B494" s="2" t="s">
         <v>1499</v>
       </c>
-      <c r="B494" s="2" t="s">
-        <v>1500</v>
-      </c>
       <c r="C494" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D494" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E494" s="2" t="s">
-        <v>1501</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="495" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A495" s="2" t="s">
+        <v>1501</v>
+      </c>
+      <c r="B495" s="2" t="s">
         <v>1502</v>
       </c>
-      <c r="B495" s="2" t="s">
-        <v>1503</v>
-      </c>
       <c r="C495" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D495" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E495" s="2" t="s">
-        <v>1504</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="496" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A496" s="2" t="s">
+        <v>1504</v>
+      </c>
+      <c r="B496" s="2" t="s">
         <v>1505</v>
       </c>
-      <c r="B496" s="2" t="s">
-        <v>1506</v>
-      </c>
       <c r="C496" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D496" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E496" s="2" t="s">
-        <v>1507</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="497" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A497" s="2" t="s">
+        <v>1507</v>
+      </c>
+      <c r="B497" s="2" t="s">
         <v>1508</v>
       </c>
-      <c r="B497" s="2" t="s">
-        <v>1509</v>
-      </c>
       <c r="C497" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D497" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E497" s="2" t="s">
-        <v>1510</v>
+        <v>1509</v>
       </c>
     </row>
     <row r="498" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A498" s="2" t="s">
+        <v>1510</v>
+      </c>
+      <c r="B498" s="2" t="s">
         <v>1511</v>
       </c>
-      <c r="B498" s="2" t="s">
-        <v>1512</v>
-      </c>
       <c r="C498" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D498" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E498" s="2" t="s">
-        <v>1513</v>
+        <v>1512</v>
       </c>
     </row>
     <row r="499" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A499" s="2" t="s">
+        <v>1513</v>
+      </c>
+      <c r="B499" s="2" t="s">
         <v>1514</v>
       </c>
-      <c r="B499" s="2" t="s">
-        <v>1515</v>
-      </c>
       <c r="C499" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D499" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E499" s="2" t="s">
-        <v>1516</v>
+        <v>1515</v>
       </c>
     </row>
     <row r="500" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A500" s="2" t="s">
+        <v>1516</v>
+      </c>
+      <c r="B500" s="2" t="s">
         <v>1517</v>
       </c>
-      <c r="B500" s="2" t="s">
-        <v>1518</v>
-      </c>
       <c r="C500" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D500" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E500" s="2" t="s">
-        <v>1519</v>
+        <v>1518</v>
       </c>
     </row>
     <row r="501" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A501" s="2" t="s">
+        <v>1519</v>
+      </c>
+      <c r="B501" s="2" t="s">
         <v>1520</v>
       </c>
-      <c r="B501" s="2" t="s">
-        <v>1521</v>
-      </c>
       <c r="C501" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D501" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E501" s="2" t="s">
-        <v>1522</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="502" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A502" s="2" t="s">
+        <v>1522</v>
+      </c>
+      <c r="B502" s="2" t="s">
         <v>1523</v>
       </c>
-      <c r="B502" s="2" t="s">
-        <v>1524</v>
-      </c>
       <c r="C502" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D502" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E502" s="2" t="s">
-        <v>1525</v>
+        <v>1524</v>
       </c>
     </row>
     <row r="503" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A503" s="2" t="s">
+        <v>1525</v>
+      </c>
+      <c r="B503" s="2" t="s">
         <v>1526</v>
       </c>
-      <c r="B503" s="2" t="s">
-        <v>1527</v>
-      </c>
       <c r="C503" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D503" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E503" s="2" t="s">
-        <v>1528</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="504" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A504" s="2" t="s">
+        <v>1528</v>
+      </c>
+      <c r="B504" s="2" t="s">
         <v>1529</v>
       </c>
-      <c r="B504" s="2" t="s">
-        <v>1530</v>
-      </c>
       <c r="C504" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D504" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E504" s="2" t="s">
-        <v>1531</v>
+        <v>1530</v>
       </c>
     </row>
     <row r="505" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A505" s="2" t="s">
+        <v>1531</v>
+      </c>
+      <c r="B505" s="2" t="s">
         <v>1532</v>
       </c>
-      <c r="B505" s="2" t="s">
-        <v>1533</v>
-      </c>
       <c r="C505" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D505" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E505" s="2" t="s">
-        <v>1534</v>
+        <v>1533</v>
       </c>
     </row>
     <row r="506" spans="1:5" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A506" s="2" t="s">
+        <v>1534</v>
+      </c>
+      <c r="B506" s="2" t="s">
         <v>1535</v>
       </c>
-      <c r="B506" s="2" t="s">
-        <v>1536</v>
-      </c>
       <c r="C506" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="D506" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E506" s="2" t="s">
-        <v>1537</v>
+        <v>1536</v>
       </c>
     </row>
   </sheetData>
@@ -14751,10 +14751,10 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>1537</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1538</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1539</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>4</v>
@@ -14765,10 +14765,10 @@
         <v>7</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>1539</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>1540</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1541</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
@@ -14776,10 +14776,10 @@
         <v>358</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>1540</v>
+        <v>1539</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>1542</v>
+        <v>1541</v>
       </c>
     </row>
     <row r="4" spans="1:3" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
@@ -14787,10 +14787,10 @@
         <v>449</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>1540</v>
+        <v>1539</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1543</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
@@ -14798,10 +14798,10 @@
         <v>540</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>1540</v>
+        <v>1539</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>1544</v>
+        <v>1543</v>
       </c>
     </row>
     <row r="6" spans="1:3" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
@@ -14809,10 +14809,10 @@
         <v>631</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>1540</v>
+        <v>1539</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1545</v>
+        <v>1544</v>
       </c>
     </row>
     <row r="7" spans="1:3" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
@@ -14820,10 +14820,10 @@
         <v>722</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>1540</v>
+        <v>1539</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>1546</v>
+        <v>1545</v>
       </c>
     </row>
     <row r="8" spans="1:3" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
@@ -14831,10 +14831,10 @@
         <v>813</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>1540</v>
+        <v>1539</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>1547</v>
+        <v>1546</v>
       </c>
     </row>
     <row r="9" spans="1:3" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
@@ -14842,76 +14842,76 @@
         <v>904</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>1540</v>
+        <v>1539</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>1548</v>
+        <v>1547</v>
       </c>
     </row>
     <row r="10" spans="1:3" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>1540</v>
+        <v>1539</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>1549</v>
+        <v>1548</v>
       </c>
     </row>
     <row r="11" spans="1:3" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>1540</v>
+        <v>1539</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>1550</v>
+        <v>1549</v>
       </c>
     </row>
     <row r="12" spans="1:3" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>1540</v>
+        <v>1539</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>1551</v>
+        <v>1550</v>
       </c>
     </row>
     <row r="13" spans="1:3" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>1540</v>
+        <v>1539</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>1552</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="14" spans="1:3" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>1540</v>
+        <v>1539</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>1553</v>
+        <v>1552</v>
       </c>
     </row>
     <row r="15" spans="1:3" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>1540</v>
+        <v>1539</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>1554</v>
+        <v>1553</v>
       </c>
     </row>
   </sheetData>
@@ -14931,12 +14931,12 @@
   <sheetData>
     <row r="1" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>1555</v>
+        <v>1554</v>
       </c>
     </row>
     <row r="2" spans="1:1" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>1556</v>
+        <v>1555</v>
       </c>
     </row>
   </sheetData>

</xml_diff>